<commit_message>
sprint 3 reparación de bugs
Se repararon bugs en la parte visual y controladores
</commit_message>
<xml_diff>
--- a/docs/Product_Backlog_ICARO_V2.xlsx
+++ b/docs/Product_Backlog_ICARO_V2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Ryzen5\Documents\Sistema_ICARO\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30698E5D-7F02-44A1-B5A3-F1F11CDA8FFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DCAE93C-1E0C-446F-9750-87D848551251}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2104,7 +2104,7 @@
     <col min="2" max="2" width="10.28515625" style="10" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.140625" style="10"/>
     <col min="4" max="4" width="84.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="84.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="73.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.5703125" style="10" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="46" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.140625" style="10"/>

</xml_diff>